<commit_message>
Renumber final bundle: Table01..Table33 (appearance order) + Fig01..Fig07, add CSV
- Tables now named TableXX.xlsx/.csv in dissertation.tex \input appearance order
  (Table01 = corpus-provenance ... Table33 = K.1); two-digit zero-padded so they
  sort correctly. Each table emits both .xlsx and .csv.
- Figures renamed FigXX.png/.pdf (Fig01..Fig07, Fig06a..Fig06d).
- collect_final_outputs.py cleans stale old-named outputs before rewriting for
  idempotent re-runs.
</commit_message>
<xml_diff>
--- a/4_outputs/final/Table10.xlsx
+++ b/4_outputs/final/Table10.xlsx
@@ -417,13 +417,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="37" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="6" customWidth="1" min="4" max="4"/>
+    <col width="7" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -434,15 +438,39 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Keyword %</t>
+          <t>Canonical</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Concept %</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr"/>
+          <t>SWD</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Chamfer</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Hausdorff</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Gauss. W_2</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Grassmann</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>linear MMD</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -452,17 +480,37 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0.4</t>
+          <t>0.191</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>0.7</t>
+          <t>0.009</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>+0.3</t>
+          <t>0.509</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>0.600</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>0.684</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>3.727</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>0.067</t>
         </is>
       </c>
     </row>
@@ -474,17 +522,37 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2.4</t>
+          <t>0.089</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>1.8</t>
+          <t>0.008</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>-0.6</t>
+          <t>0.388</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>0.454</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>0.618</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>3.629</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>0.057</t>
         </is>
       </c>
     </row>
@@ -496,17 +564,37 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>25.7</t>
+          <t>0.319</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>25.7</t>
+          <t>0.011</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>-0.0</t>
+          <t>0.454</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>0.581</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>0.717</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>3.717</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>0.129</t>
         </is>
       </c>
     </row>
@@ -518,17 +606,37 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>15.6</t>
+          <t>0.158</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>8.3</t>
+          <t>0.010</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>-7.3</t>
+          <t>0.399</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>0.487</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>0.607</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>3.307</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>0.096</t>
         </is>
       </c>
     </row>
@@ -540,17 +648,37 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2.0</t>
+          <t>0.151</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>1.7</t>
+          <t>0.010</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>-0.2</t>
+          <t>0.429</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>0.529</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>0.646</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>3.514</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>0.095</t>
         </is>
       </c>
     </row>
@@ -562,17 +690,37 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>0.130</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>0.8</t>
+          <t>0.009</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>-0.2</t>
+          <t>0.417</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>0.475</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>0.639</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>3.598</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>0.080</t>
         </is>
       </c>
     </row>
@@ -584,17 +732,37 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>4.1</t>
+          <t>0.170</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>0.010</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>+0.6</t>
+          <t>0.427</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>0.522</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>0.687</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>3.729</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>0.105</t>
         </is>
       </c>
     </row>
@@ -606,17 +774,37 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2.2</t>
+          <t>0.184</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2.3</t>
+          <t>0.008</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>+0.1</t>
+          <t>0.474</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>0.564</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>0.658</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>3.566</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>0.065</t>
         </is>
       </c>
     </row>
@@ -628,17 +816,37 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>20.1</t>
+          <t>0.228</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>25.9</t>
+          <t>0.010</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>+5.8</t>
+          <t>0.430</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>0.556</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>0.671</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>3.444</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>0.104</t>
         </is>
       </c>
     </row>
@@ -650,17 +858,37 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>0.9</t>
+          <t>0.195</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>0.8</t>
+          <t>0.008</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>-0.1</t>
+          <t>0.456</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>0.517</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>0.617</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>3.343</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>0.062</t>
         </is>
       </c>
     </row>
@@ -672,17 +900,37 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>5.1</t>
+          <t>0.209</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>8.0</t>
+          <t>0.009</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>+2.9</t>
+          <t>0.446</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>0.542</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>0.677</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>3.484</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>0.091</t>
         </is>
       </c>
     </row>
@@ -694,17 +942,37 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>0.156</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2.7</t>
+          <t>0.009</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>+1.2</t>
+          <t>0.467</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>0.566</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>0.677</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>3.462</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>0.094</t>
         </is>
       </c>
     </row>
@@ -716,17 +984,37 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>3.7</t>
+          <t>0.219</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>4.2</t>
+          <t>0.010</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>+0.5</t>
+          <t>0.417</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>0.498</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>0.667</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>3.667</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>0.117</t>
         </is>
       </c>
     </row>
@@ -738,17 +1026,37 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>1.6</t>
+          <t>0.132</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>1.3</t>
+          <t>0.010</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>-0.3</t>
+          <t>0.415</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>0.510</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>0.675</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>3.753</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>0.098</t>
         </is>
       </c>
     </row>
@@ -760,17 +1068,37 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2.2</t>
+          <t>0.084</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2.1</t>
+          <t>0.008</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>-0.1</t>
+          <t>0.394</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>0.464</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>0.578</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>3.421</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>0.056</t>
         </is>
       </c>
     </row>
@@ -782,17 +1110,37 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>11.2</t>
+          <t>0.242</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>8.8</t>
+          <t>0.010</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>-2.4</t>
+          <t>0.417</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>0.520</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>0.640</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>3.333</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>0.103</t>
         </is>
       </c>
     </row>
@@ -804,29 +1152,81 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>0.3</t>
+          <t>0.326</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>0.2</t>
+          <t>0.009</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>-0.0</t>
+          <t>0.461</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>0.490</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>0.595</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>2.993</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>0.104</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Spearman ρ = 0.948; Kendall = 0.868</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr"/>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr"/>
+          <t>ρ vs. canonical</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>0.525</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>0.485</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>0.444</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>0.243</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>-0.243</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>0.620</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>